<commit_message>
Add .gitignore file and remove Excel temporary files
</commit_message>
<xml_diff>
--- a/excel/medical-parts-analysis.xlsx
+++ b/excel/medical-parts-analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jeremy\source\repos\nosirrah01\medical-parts-data-analysis\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{08FC09E6-0957-424E-B6E0-9B8939305ED7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{91F8C394-8468-4C11-9A56-431623BFDA87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="21690" xr2:uid="{3D9AE382-BE39-4EE9-A057-74AE2767EA6F}"/>
   </bookViews>
@@ -4849,7 +4849,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{13A7A260-AA38-4A66-87D0-36E39FC2254D}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="6">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{13A7A260-AA38-4A66-87D0-36E39FC2254D}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
   <location ref="A3:B10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="17">
     <pivotField showAll="0"/>

</xml_diff>

<commit_message>
Update medical parts analysis Excel file with new data
</commit_message>
<xml_diff>
--- a/excel/medical-parts-analysis.xlsx
+++ b/excel/medical-parts-analysis.xlsx
@@ -8,19 +8,32 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Jeremy\source\repos\nosirrah01\medical-parts-data-analysis\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{91F8C394-8468-4C11-9A56-431623BFDA87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{166375FB-3778-4CFE-8DD7-98CDAB6056A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="21690" xr2:uid="{3D9AE382-BE39-4EE9-A057-74AE2767EA6F}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="21690" activeTab="2" xr2:uid="{3D9AE382-BE39-4EE9-A057-74AE2767EA6F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="3" r:id="rId2"/>
     <sheet name="orders_raw" sheetId="1" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="5" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -316,6 +329,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
+  </numFmts>
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -793,14 +809,13 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -848,13 +863,13 @@
   </cellStyles>
   <dxfs count="3">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -965,19 +980,7 @@
           <a:effectLst/>
         </c:spPr>
         <c:marker>
-          <c:symbol val="circle"/>
-          <c:size val="5"/>
-          <c:spPr>
-            <a:solidFill>
-              <a:schemeClr val="accent1"/>
-            </a:solidFill>
-            <a:ln w="9525">
-              <a:solidFill>
-                <a:schemeClr val="accent1"/>
-              </a:solidFill>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
+          <c:symbol val="none"/>
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
@@ -1207,7 +1210,7 @@
           <a:effectLst/>
         </c:spPr>
         <c:txPr>
-          <a:bodyPr rot="-2100000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:bodyPr rot="-2100000" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
           <a:lstStyle/>
           <a:p>
             <a:pPr>
@@ -4849,7 +4852,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{13A7A260-AA38-4A66-87D0-36E39FC2254D}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{13A7A260-AA38-4A66-87D0-36E39FC2254D}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="9">
   <location ref="A3:B10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="17">
     <pivotField showAll="0"/>
@@ -4945,7 +4948,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F86A53AF-39E3-4DA8-A4A7-7C87F2DF88F4}" name="PivotTable2" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F86A53AF-39E3-4DA8-A4A7-7C87F2DF88F4}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:C8" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="17">
     <pivotField dataField="1" showAll="0"/>
@@ -5026,7 +5029,7 @@
   <autoFilter ref="A1:Q151" xr:uid="{3EE8128A-0022-4BEB-BB3F-4C617BDDFBBA}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{9B8E0011-6781-4139-9A44-8F844BE1AB82}" name="OrderID"/>
-    <tableColumn id="2" xr3:uid="{16C1D808-5389-4983-A2E5-B1AC38267666}" name="OrderDate" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{16C1D808-5389-4983-A2E5-B1AC38267666}" name="OrderDate" dataDxfId="0"/>
     <tableColumn id="3" xr3:uid="{4897CCA7-E26E-4D05-891B-65119BE1B4F6}" name="CustomerID"/>
     <tableColumn id="4" xr3:uid="{0E0FDD0D-6DBE-4713-8B3C-B072E8F19B51}" name="CustomerName"/>
     <tableColumn id="5" xr3:uid="{1FC8C3D0-4570-4E4C-BF66-10085D7FA9B6}" name="Region"/>
@@ -5040,10 +5043,10 @@
     <tableColumn id="13" xr3:uid="{8FEC794C-CDAF-4263-B9D7-BD8978BA6C39}" name="ShippingDays"/>
     <tableColumn id="14" xr3:uid="{02554CDF-851B-4E0A-8493-0EE645AEA97B}" name="RushOrder"/>
     <tableColumn id="15" xr3:uid="{3EA11F9E-CAD9-4CE8-AFC4-D75955107E20}" name="Returned"/>
-    <tableColumn id="16" xr3:uid="{EA1F5B72-5AA6-4A16-8C31-BF1EF6699CD1}" name="Revenue" dataDxfId="1">
+    <tableColumn id="16" xr3:uid="{EA1F5B72-5AA6-4A16-8C31-BF1EF6699CD1}" name="Revenue" dataDxfId="2">
       <calculatedColumnFormula>Table1[[#This Row],[Quantity]]*Table1[[#This Row],[UnitPrice]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{1E27B0D1-B448-4861-AAC9-20981F19EA41}" name="ShippingStatus" dataDxfId="0">
+    <tableColumn id="17" xr3:uid="{1E27B0D1-B448-4861-AAC9-20981F19EA41}" name="ShippingStatus" dataDxfId="1">
       <calculatedColumnFormula>IF(Table1[[#This Row],[ShippingDays]]&gt;Table1[[#This Row],[ExpectedShippingDays]],"Late","On Time")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5376,7 +5379,7 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>90</v>
       </c>
       <c r="B3" t="s">
@@ -5384,58 +5387,58 @@
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4">
         <v>75825</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5">
         <v>44295</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6">
         <v>32885</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7">
         <v>32380</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8">
         <v>12985</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9">
         <v>10920</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10">
         <v>209290</v>
       </c>
     </row>
@@ -5456,7 +5459,7 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>90</v>
       </c>
       <c r="B3" t="s">
@@ -5467,57 +5470,57 @@
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4">
         <v>52</v>
       </c>
-      <c r="C4" s="4">
+      <c r="C4">
         <v>3.2884615384615383</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5">
         <v>35</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5">
         <v>3.2285714285714286</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6">
         <v>38</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C6">
         <v>3.3947368421052633</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7">
         <v>25</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7">
         <v>3.52</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
+      <c r="A8" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8">
         <v>150</v>
       </c>
-      <c r="C8" s="4">
+      <c r="C8">
         <v>3.34</v>
       </c>
     </row>
@@ -5532,7 +5535,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.26953125" customWidth="1"/>
-    <col min="2" max="2" width="11.36328125" customWidth="1"/>
+    <col min="2" max="2" width="11.36328125" style="3" customWidth="1"/>
     <col min="3" max="3" width="12.81640625" customWidth="1"/>
     <col min="4" max="4" width="15.90625" customWidth="1"/>
     <col min="6" max="6" width="11.1796875" customWidth="1"/>
@@ -5553,7 +5556,7 @@
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
@@ -5606,7 +5609,7 @@
       <c r="A2">
         <v>1026</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="3">
         <v>46024</v>
       </c>
       <c r="C2" t="s">
@@ -5661,7 +5664,7 @@
       <c r="A3">
         <v>1013</v>
       </c>
-      <c r="B3" s="1">
+      <c r="B3" s="3">
         <v>46026</v>
       </c>
       <c r="C3" t="s">
@@ -5716,7 +5719,7 @@
       <c r="A4">
         <v>1025</v>
       </c>
-      <c r="B4" s="1">
+      <c r="B4" s="3">
         <v>46027</v>
       </c>
       <c r="C4" t="s">
@@ -5771,7 +5774,7 @@
       <c r="A5">
         <v>1078</v>
       </c>
-      <c r="B5" s="1">
+      <c r="B5" s="3">
         <v>46027</v>
       </c>
       <c r="C5" t="s">
@@ -5826,7 +5829,7 @@
       <c r="A6">
         <v>1125</v>
       </c>
-      <c r="B6" s="1">
+      <c r="B6" s="3">
         <v>46028</v>
       </c>
       <c r="C6" t="s">
@@ -5881,7 +5884,7 @@
       <c r="A7">
         <v>1009</v>
       </c>
-      <c r="B7" s="1">
+      <c r="B7" s="3">
         <v>46032</v>
       </c>
       <c r="C7" t="s">
@@ -5936,7 +5939,7 @@
       <c r="A8">
         <v>1038</v>
       </c>
-      <c r="B8" s="1">
+      <c r="B8" s="3">
         <v>46034</v>
       </c>
       <c r="C8" t="s">
@@ -5991,7 +5994,7 @@
       <c r="A9">
         <v>1067</v>
       </c>
-      <c r="B9" s="1">
+      <c r="B9" s="3">
         <v>46034</v>
       </c>
       <c r="C9" t="s">
@@ -6046,7 +6049,7 @@
       <c r="A10">
         <v>1099</v>
       </c>
-      <c r="B10" s="1">
+      <c r="B10" s="3">
         <v>46035</v>
       </c>
       <c r="C10" t="s">
@@ -6101,7 +6104,7 @@
       <c r="A11">
         <v>1057</v>
       </c>
-      <c r="B11" s="1">
+      <c r="B11" s="3">
         <v>46039</v>
       </c>
       <c r="C11" t="s">
@@ -6156,7 +6159,7 @@
       <c r="A12">
         <v>1006</v>
       </c>
-      <c r="B12" s="1">
+      <c r="B12" s="3">
         <v>46041</v>
       </c>
       <c r="C12" t="s">
@@ -6211,7 +6214,7 @@
       <c r="A13">
         <v>1031</v>
       </c>
-      <c r="B13" s="1">
+      <c r="B13" s="3">
         <v>46042</v>
       </c>
       <c r="C13" t="s">
@@ -6266,7 +6269,7 @@
       <c r="A14">
         <v>1101</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14" s="3">
         <v>46043</v>
       </c>
       <c r="C14" t="s">
@@ -6321,7 +6324,7 @@
       <c r="A15">
         <v>1080</v>
       </c>
-      <c r="B15" s="1">
+      <c r="B15" s="3">
         <v>46045</v>
       </c>
       <c r="C15" t="s">
@@ -6376,7 +6379,7 @@
       <c r="A16">
         <v>1002</v>
       </c>
-      <c r="B16" s="1">
+      <c r="B16" s="3">
         <v>46046</v>
       </c>
       <c r="C16" t="s">
@@ -6431,7 +6434,7 @@
       <c r="A17">
         <v>1070</v>
       </c>
-      <c r="B17" s="1">
+      <c r="B17" s="3">
         <v>46046</v>
       </c>
       <c r="C17" t="s">
@@ -6486,7 +6489,7 @@
       <c r="A18">
         <v>1138</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B18" s="3">
         <v>46047</v>
       </c>
       <c r="C18" t="s">
@@ -6541,7 +6544,7 @@
       <c r="A19">
         <v>1104</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B19" s="3">
         <v>46049</v>
       </c>
       <c r="C19" t="s">
@@ -6596,7 +6599,7 @@
       <c r="A20">
         <v>1034</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B20" s="3">
         <v>46051</v>
       </c>
       <c r="C20" t="s">
@@ -6651,7 +6654,7 @@
       <c r="A21">
         <v>1052</v>
       </c>
-      <c r="B21" s="1">
+      <c r="B21" s="3">
         <v>46051</v>
       </c>
       <c r="C21" t="s">
@@ -6706,7 +6709,7 @@
       <c r="A22">
         <v>1065</v>
       </c>
-      <c r="B22" s="1">
+      <c r="B22" s="3">
         <v>46053</v>
       </c>
       <c r="C22" t="s">
@@ -6761,7 +6764,7 @@
       <c r="A23">
         <v>1079</v>
       </c>
-      <c r="B23" s="1">
+      <c r="B23" s="3">
         <v>46053</v>
       </c>
       <c r="C23" t="s">
@@ -6816,7 +6819,7 @@
       <c r="A24">
         <v>1091</v>
       </c>
-      <c r="B24" s="1">
+      <c r="B24" s="3">
         <v>46053</v>
       </c>
       <c r="C24" t="s">
@@ -6871,7 +6874,7 @@
       <c r="A25">
         <v>1064</v>
       </c>
-      <c r="B25" s="1">
+      <c r="B25" s="3">
         <v>46056</v>
       </c>
       <c r="C25" t="s">
@@ -6926,7 +6929,7 @@
       <c r="A26">
         <v>1112</v>
       </c>
-      <c r="B26" s="1">
+      <c r="B26" s="3">
         <v>46057</v>
       </c>
       <c r="C26" t="s">
@@ -6981,7 +6984,7 @@
       <c r="A27">
         <v>1096</v>
       </c>
-      <c r="B27" s="1">
+      <c r="B27" s="3">
         <v>46058</v>
       </c>
       <c r="C27" t="s">
@@ -7036,7 +7039,7 @@
       <c r="A28">
         <v>1118</v>
       </c>
-      <c r="B28" s="1">
+      <c r="B28" s="3">
         <v>46059</v>
       </c>
       <c r="C28" t="s">
@@ -7091,7 +7094,7 @@
       <c r="A29">
         <v>1142</v>
       </c>
-      <c r="B29" s="1">
+      <c r="B29" s="3">
         <v>46059</v>
       </c>
       <c r="C29" t="s">
@@ -7146,7 +7149,7 @@
       <c r="A30">
         <v>1085</v>
       </c>
-      <c r="B30" s="1">
+      <c r="B30" s="3">
         <v>46060</v>
       </c>
       <c r="C30" t="s">
@@ -7201,7 +7204,7 @@
       <c r="A31">
         <v>1124</v>
       </c>
-      <c r="B31" s="1">
+      <c r="B31" s="3">
         <v>46061</v>
       </c>
       <c r="C31" t="s">
@@ -7256,7 +7259,7 @@
       <c r="A32">
         <v>1037</v>
       </c>
-      <c r="B32" s="1">
+      <c r="B32" s="3">
         <v>46062</v>
       </c>
       <c r="C32" t="s">
@@ -7311,7 +7314,7 @@
       <c r="A33">
         <v>1056</v>
       </c>
-      <c r="B33" s="1">
+      <c r="B33" s="3">
         <v>46062</v>
       </c>
       <c r="C33" t="s">
@@ -7366,7 +7369,7 @@
       <c r="A34">
         <v>1012</v>
       </c>
-      <c r="B34" s="1">
+      <c r="B34" s="3">
         <v>46064</v>
       </c>
       <c r="C34" t="s">
@@ -7421,7 +7424,7 @@
       <c r="A35">
         <v>1008</v>
       </c>
-      <c r="B35" s="1">
+      <c r="B35" s="3">
         <v>46065</v>
       </c>
       <c r="C35" t="s">
@@ -7476,7 +7479,7 @@
       <c r="A36">
         <v>1049</v>
       </c>
-      <c r="B36" s="1">
+      <c r="B36" s="3">
         <v>46067</v>
       </c>
       <c r="C36" t="s">
@@ -7531,7 +7534,7 @@
       <c r="A37">
         <v>1066</v>
       </c>
-      <c r="B37" s="1">
+      <c r="B37" s="3">
         <v>46074</v>
       </c>
       <c r="C37" t="s">
@@ -7586,7 +7589,7 @@
       <c r="A38">
         <v>1041</v>
       </c>
-      <c r="B38" s="1">
+      <c r="B38" s="3">
         <v>46075</v>
       </c>
       <c r="C38" t="s">
@@ -7641,7 +7644,7 @@
       <c r="A39">
         <v>1048</v>
       </c>
-      <c r="B39" s="1">
+      <c r="B39" s="3">
         <v>46077</v>
       </c>
       <c r="C39" t="s">
@@ -7696,7 +7699,7 @@
       <c r="A40">
         <v>1082</v>
       </c>
-      <c r="B40" s="1">
+      <c r="B40" s="3">
         <v>46077</v>
       </c>
       <c r="C40" t="s">
@@ -7751,7 +7754,7 @@
       <c r="A41">
         <v>1018</v>
       </c>
-      <c r="B41" s="1">
+      <c r="B41" s="3">
         <v>46078</v>
       </c>
       <c r="C41" t="s">
@@ -7806,7 +7809,7 @@
       <c r="A42">
         <v>1027</v>
       </c>
-      <c r="B42" s="1">
+      <c r="B42" s="3">
         <v>46079</v>
       </c>
       <c r="C42" t="s">
@@ -7861,7 +7864,7 @@
       <c r="A43">
         <v>1094</v>
       </c>
-      <c r="B43" s="1">
+      <c r="B43" s="3">
         <v>46081</v>
       </c>
       <c r="C43" t="s">
@@ -7916,7 +7919,7 @@
       <c r="A44">
         <v>1075</v>
       </c>
-      <c r="B44" s="1">
+      <c r="B44" s="3">
         <v>46088</v>
       </c>
       <c r="C44" t="s">
@@ -7971,7 +7974,7 @@
       <c r="A45">
         <v>1030</v>
       </c>
-      <c r="B45" s="1">
+      <c r="B45" s="3">
         <v>46090</v>
       </c>
       <c r="C45" t="s">
@@ -8026,7 +8029,7 @@
       <c r="A46">
         <v>1043</v>
       </c>
-      <c r="B46" s="1">
+      <c r="B46" s="3">
         <v>46090</v>
       </c>
       <c r="C46" t="s">
@@ -8081,7 +8084,7 @@
       <c r="A47">
         <v>1014</v>
       </c>
-      <c r="B47" s="1">
+      <c r="B47" s="3">
         <v>46091</v>
       </c>
       <c r="C47" t="s">
@@ -8136,7 +8139,7 @@
       <c r="A48">
         <v>1035</v>
       </c>
-      <c r="B48" s="1">
+      <c r="B48" s="3">
         <v>46091</v>
       </c>
       <c r="C48" t="s">
@@ -8191,7 +8194,7 @@
       <c r="A49">
         <v>1036</v>
       </c>
-      <c r="B49" s="1">
+      <c r="B49" s="3">
         <v>46091</v>
       </c>
       <c r="C49" t="s">
@@ -8246,7 +8249,7 @@
       <c r="A50">
         <v>1088</v>
       </c>
-      <c r="B50" s="1">
+      <c r="B50" s="3">
         <v>46092</v>
       </c>
       <c r="C50" t="s">
@@ -8301,7 +8304,7 @@
       <c r="A51">
         <v>1095</v>
       </c>
-      <c r="B51" s="1">
+      <c r="B51" s="3">
         <v>46093</v>
       </c>
       <c r="C51" t="s">
@@ -8356,7 +8359,7 @@
       <c r="A52">
         <v>1004</v>
       </c>
-      <c r="B52" s="1">
+      <c r="B52" s="3">
         <v>46095</v>
       </c>
       <c r="C52" t="s">
@@ -8411,7 +8414,7 @@
       <c r="A53">
         <v>1042</v>
       </c>
-      <c r="B53" s="1">
+      <c r="B53" s="3">
         <v>46095</v>
       </c>
       <c r="C53" t="s">
@@ -8466,7 +8469,7 @@
       <c r="A54">
         <v>1114</v>
       </c>
-      <c r="B54" s="1">
+      <c r="B54" s="3">
         <v>46099</v>
       </c>
       <c r="C54" t="s">
@@ -8521,7 +8524,7 @@
       <c r="A55">
         <v>1046</v>
       </c>
-      <c r="B55" s="1">
+      <c r="B55" s="3">
         <v>46100</v>
       </c>
       <c r="C55" t="s">
@@ -8576,7 +8579,7 @@
       <c r="A56">
         <v>1086</v>
       </c>
-      <c r="B56" s="1">
+      <c r="B56" s="3">
         <v>46101</v>
       </c>
       <c r="C56" t="s">
@@ -8631,7 +8634,7 @@
       <c r="A57">
         <v>1150</v>
       </c>
-      <c r="B57" s="1">
+      <c r="B57" s="3">
         <v>46101</v>
       </c>
       <c r="C57" t="s">
@@ -8686,7 +8689,7 @@
       <c r="A58">
         <v>1016</v>
       </c>
-      <c r="B58" s="1">
+      <c r="B58" s="3">
         <v>46102</v>
       </c>
       <c r="C58" t="s">
@@ -8741,7 +8744,7 @@
       <c r="A59">
         <v>1146</v>
       </c>
-      <c r="B59" s="1">
+      <c r="B59" s="3">
         <v>46103</v>
       </c>
       <c r="C59" t="s">
@@ -8796,7 +8799,7 @@
       <c r="A60">
         <v>1087</v>
       </c>
-      <c r="B60" s="1">
+      <c r="B60" s="3">
         <v>46106</v>
       </c>
       <c r="C60" t="s">
@@ -8851,7 +8854,7 @@
       <c r="A61">
         <v>1071</v>
       </c>
-      <c r="B61" s="1">
+      <c r="B61" s="3">
         <v>46107</v>
       </c>
       <c r="C61" t="s">
@@ -8906,7 +8909,7 @@
       <c r="A62">
         <v>1129</v>
       </c>
-      <c r="B62" s="1">
+      <c r="B62" s="3">
         <v>46107</v>
       </c>
       <c r="C62" t="s">
@@ -8961,7 +8964,7 @@
       <c r="A63">
         <v>1040</v>
       </c>
-      <c r="B63" s="1">
+      <c r="B63" s="3">
         <v>46109</v>
       </c>
       <c r="C63" t="s">
@@ -9016,7 +9019,7 @@
       <c r="A64">
         <v>1062</v>
       </c>
-      <c r="B64" s="1">
+      <c r="B64" s="3">
         <v>46110</v>
       </c>
       <c r="C64" t="s">
@@ -9071,7 +9074,7 @@
       <c r="A65">
         <v>1137</v>
       </c>
-      <c r="B65" s="1">
+      <c r="B65" s="3">
         <v>46110</v>
       </c>
       <c r="C65" t="s">
@@ -9126,7 +9129,7 @@
       <c r="A66">
         <v>1032</v>
       </c>
-      <c r="B66" s="1">
+      <c r="B66" s="3">
         <v>46113</v>
       </c>
       <c r="C66" t="s">
@@ -9181,7 +9184,7 @@
       <c r="A67">
         <v>1063</v>
       </c>
-      <c r="B67" s="1">
+      <c r="B67" s="3">
         <v>46113</v>
       </c>
       <c r="C67" t="s">
@@ -9236,7 +9239,7 @@
       <c r="A68">
         <v>1147</v>
       </c>
-      <c r="B68" s="1">
+      <c r="B68" s="3">
         <v>46113</v>
       </c>
       <c r="C68" t="s">
@@ -9291,7 +9294,7 @@
       <c r="A69">
         <v>1011</v>
       </c>
-      <c r="B69" s="1">
+      <c r="B69" s="3">
         <v>46116</v>
       </c>
       <c r="C69" t="s">
@@ -9346,7 +9349,7 @@
       <c r="A70">
         <v>1068</v>
       </c>
-      <c r="B70" s="1">
+      <c r="B70" s="3">
         <v>46116</v>
       </c>
       <c r="C70" t="s">
@@ -9401,7 +9404,7 @@
       <c r="A71">
         <v>1126</v>
       </c>
-      <c r="B71" s="1">
+      <c r="B71" s="3">
         <v>46116</v>
       </c>
       <c r="C71" t="s">
@@ -9456,7 +9459,7 @@
       <c r="A72">
         <v>1007</v>
       </c>
-      <c r="B72" s="1">
+      <c r="B72" s="3">
         <v>46117</v>
       </c>
       <c r="C72" t="s">
@@ -9511,7 +9514,7 @@
       <c r="A73">
         <v>1113</v>
       </c>
-      <c r="B73" s="1">
+      <c r="B73" s="3">
         <v>46117</v>
       </c>
       <c r="C73" t="s">
@@ -9566,7 +9569,7 @@
       <c r="A74">
         <v>1015</v>
       </c>
-      <c r="B74" s="1">
+      <c r="B74" s="3">
         <v>46119</v>
       </c>
       <c r="C74" t="s">
@@ -9621,7 +9624,7 @@
       <c r="A75">
         <v>1047</v>
       </c>
-      <c r="B75" s="1">
+      <c r="B75" s="3">
         <v>46121</v>
       </c>
       <c r="C75" t="s">
@@ -9676,7 +9679,7 @@
       <c r="A76">
         <v>1010</v>
       </c>
-      <c r="B76" s="1">
+      <c r="B76" s="3">
         <v>46125</v>
       </c>
       <c r="C76" t="s">
@@ -9731,7 +9734,7 @@
       <c r="A77">
         <v>1023</v>
       </c>
-      <c r="B77" s="1">
+      <c r="B77" s="3">
         <v>46127</v>
       </c>
       <c r="C77" t="s">
@@ -9786,7 +9789,7 @@
       <c r="A78">
         <v>1060</v>
       </c>
-      <c r="B78" s="1">
+      <c r="B78" s="3">
         <v>46127</v>
       </c>
       <c r="C78" t="s">
@@ -9841,7 +9844,7 @@
       <c r="A79">
         <v>1090</v>
       </c>
-      <c r="B79" s="1">
+      <c r="B79" s="3">
         <v>46129</v>
       </c>
       <c r="C79" t="s">
@@ -9896,7 +9899,7 @@
       <c r="A80">
         <v>1051</v>
       </c>
-      <c r="B80" s="1">
+      <c r="B80" s="3">
         <v>46130</v>
       </c>
       <c r="C80" t="s">
@@ -9951,7 +9954,7 @@
       <c r="A81">
         <v>1022</v>
       </c>
-      <c r="B81" s="1">
+      <c r="B81" s="3">
         <v>46134</v>
       </c>
       <c r="C81" t="s">
@@ -10006,7 +10009,7 @@
       <c r="A82">
         <v>1105</v>
       </c>
-      <c r="B82" s="1">
+      <c r="B82" s="3">
         <v>46134</v>
       </c>
       <c r="C82" t="s">
@@ -10061,7 +10064,7 @@
       <c r="A83">
         <v>1081</v>
       </c>
-      <c r="B83" s="1">
+      <c r="B83" s="3">
         <v>46137</v>
       </c>
       <c r="C83" t="s">
@@ -10116,7 +10119,7 @@
       <c r="A84">
         <v>1128</v>
       </c>
-      <c r="B84" s="1">
+      <c r="B84" s="3">
         <v>46137</v>
       </c>
       <c r="C84" t="s">
@@ -10171,7 +10174,7 @@
       <c r="A85">
         <v>1108</v>
       </c>
-      <c r="B85" s="1">
+      <c r="B85" s="3">
         <v>46140</v>
       </c>
       <c r="C85" t="s">
@@ -10226,7 +10229,7 @@
       <c r="A86">
         <v>1119</v>
       </c>
-      <c r="B86" s="1">
+      <c r="B86" s="3">
         <v>46140</v>
       </c>
       <c r="C86" t="s">
@@ -10281,7 +10284,7 @@
       <c r="A87">
         <v>1131</v>
       </c>
-      <c r="B87" s="1">
+      <c r="B87" s="3">
         <v>46140</v>
       </c>
       <c r="C87" t="s">
@@ -10336,7 +10339,7 @@
       <c r="A88">
         <v>1005</v>
       </c>
-      <c r="B88" s="1">
+      <c r="B88" s="3">
         <v>46141</v>
       </c>
       <c r="C88" t="s">
@@ -10391,7 +10394,7 @@
       <c r="A89">
         <v>1024</v>
       </c>
-      <c r="B89" s="1">
+      <c r="B89" s="3">
         <v>46142</v>
       </c>
       <c r="C89" t="s">
@@ -10446,7 +10449,7 @@
       <c r="A90">
         <v>1053</v>
       </c>
-      <c r="B90" s="1">
+      <c r="B90" s="3">
         <v>46142</v>
       </c>
       <c r="C90" t="s">
@@ -10501,7 +10504,7 @@
       <c r="A91">
         <v>1107</v>
       </c>
-      <c r="B91" s="1">
+      <c r="B91" s="3">
         <v>46143</v>
       </c>
       <c r="C91" t="s">
@@ -10556,7 +10559,7 @@
       <c r="A92">
         <v>1083</v>
       </c>
-      <c r="B92" s="1">
+      <c r="B92" s="3">
         <v>46144</v>
       </c>
       <c r="C92" t="s">
@@ -10611,7 +10614,7 @@
       <c r="A93">
         <v>1074</v>
       </c>
-      <c r="B93" s="1">
+      <c r="B93" s="3">
         <v>46145</v>
       </c>
       <c r="C93" t="s">
@@ -10666,7 +10669,7 @@
       <c r="A94">
         <v>1132</v>
       </c>
-      <c r="B94" s="1">
+      <c r="B94" s="3">
         <v>46145</v>
       </c>
       <c r="C94" t="s">
@@ -10721,7 +10724,7 @@
       <c r="A95">
         <v>1076</v>
       </c>
-      <c r="B95" s="1">
+      <c r="B95" s="3">
         <v>46147</v>
       </c>
       <c r="C95" t="s">
@@ -10776,7 +10779,7 @@
       <c r="A96">
         <v>1055</v>
       </c>
-      <c r="B96" s="1">
+      <c r="B96" s="3">
         <v>46148</v>
       </c>
       <c r="C96" t="s">
@@ -10831,7 +10834,7 @@
       <c r="A97">
         <v>1093</v>
       </c>
-      <c r="B97" s="1">
+      <c r="B97" s="3">
         <v>46148</v>
       </c>
       <c r="C97" t="s">
@@ -10886,7 +10889,7 @@
       <c r="A98">
         <v>1073</v>
       </c>
-      <c r="B98" s="1">
+      <c r="B98" s="3">
         <v>46149</v>
       </c>
       <c r="C98" t="s">
@@ -10941,7 +10944,7 @@
       <c r="A99">
         <v>1044</v>
       </c>
-      <c r="B99" s="1">
+      <c r="B99" s="3">
         <v>46154</v>
       </c>
       <c r="C99" t="s">
@@ -10996,7 +10999,7 @@
       <c r="A100">
         <v>1019</v>
       </c>
-      <c r="B100" s="1">
+      <c r="B100" s="3">
         <v>46156</v>
       </c>
       <c r="C100" t="s">
@@ -11051,7 +11054,7 @@
       <c r="A101">
         <v>1127</v>
       </c>
-      <c r="B101" s="1">
+      <c r="B101" s="3">
         <v>46157</v>
       </c>
       <c r="C101" t="s">
@@ -11106,7 +11109,7 @@
       <c r="A102">
         <v>1028</v>
       </c>
-      <c r="B102" s="1">
+      <c r="B102" s="3">
         <v>46159</v>
       </c>
       <c r="C102" t="s">
@@ -11161,7 +11164,7 @@
       <c r="A103">
         <v>1017</v>
       </c>
-      <c r="B103" s="1">
+      <c r="B103" s="3">
         <v>46160</v>
       </c>
       <c r="C103" t="s">
@@ -11216,7 +11219,7 @@
       <c r="A104">
         <v>1077</v>
       </c>
-      <c r="B104" s="1">
+      <c r="B104" s="3">
         <v>46160</v>
       </c>
       <c r="C104" t="s">
@@ -11271,7 +11274,7 @@
       <c r="A105">
         <v>1102</v>
       </c>
-      <c r="B105" s="1">
+      <c r="B105" s="3">
         <v>46160</v>
       </c>
       <c r="C105" t="s">
@@ -11326,7 +11329,7 @@
       <c r="A106">
         <v>1021</v>
       </c>
-      <c r="B106" s="1">
+      <c r="B106" s="3">
         <v>46162</v>
       </c>
       <c r="C106" t="s">
@@ -11381,7 +11384,7 @@
       <c r="A107">
         <v>1003</v>
       </c>
-      <c r="B107" s="1">
+      <c r="B107" s="3">
         <v>46163</v>
       </c>
       <c r="C107" t="s">
@@ -11436,7 +11439,7 @@
       <c r="A108">
         <v>1059</v>
       </c>
-      <c r="B108" s="1">
+      <c r="B108" s="3">
         <v>46163</v>
       </c>
       <c r="C108" t="s">
@@ -11491,7 +11494,7 @@
       <c r="A109">
         <v>1098</v>
       </c>
-      <c r="B109" s="1">
+      <c r="B109" s="3">
         <v>46163</v>
       </c>
       <c r="C109" t="s">
@@ -11546,7 +11549,7 @@
       <c r="A110">
         <v>1054</v>
       </c>
-      <c r="B110" s="1">
+      <c r="B110" s="3">
         <v>46164</v>
       </c>
       <c r="C110" t="s">
@@ -11601,7 +11604,7 @@
       <c r="A111">
         <v>1123</v>
       </c>
-      <c r="B111" s="1">
+      <c r="B111" s="3">
         <v>46165</v>
       </c>
       <c r="C111" t="s">
@@ -11656,7 +11659,7 @@
       <c r="A112">
         <v>1072</v>
       </c>
-      <c r="B112" s="1">
+      <c r="B112" s="3">
         <v>46166</v>
       </c>
       <c r="C112" t="s">
@@ -11711,7 +11714,7 @@
       <c r="A113">
         <v>1135</v>
       </c>
-      <c r="B113" s="1">
+      <c r="B113" s="3">
         <v>46166</v>
       </c>
       <c r="C113" t="s">
@@ -11766,7 +11769,7 @@
       <c r="A114">
         <v>1117</v>
       </c>
-      <c r="B114" s="1">
+      <c r="B114" s="3">
         <v>46167</v>
       </c>
       <c r="C114" t="s">
@@ -11821,7 +11824,7 @@
       <c r="A115">
         <v>1133</v>
       </c>
-      <c r="B115" s="1">
+      <c r="B115" s="3">
         <v>46167</v>
       </c>
       <c r="C115" t="s">
@@ -11876,7 +11879,7 @@
       <c r="A116">
         <v>1149</v>
       </c>
-      <c r="B116" s="1">
+      <c r="B116" s="3">
         <v>46168</v>
       </c>
       <c r="C116" t="s">
@@ -11931,7 +11934,7 @@
       <c r="A117">
         <v>1029</v>
       </c>
-      <c r="B117" s="1">
+      <c r="B117" s="3">
         <v>46169</v>
       </c>
       <c r="C117" t="s">
@@ -11986,7 +11989,7 @@
       <c r="A118">
         <v>1139</v>
       </c>
-      <c r="B118" s="1">
+      <c r="B118" s="3">
         <v>46169</v>
       </c>
       <c r="C118" t="s">
@@ -12041,7 +12044,7 @@
       <c r="A119">
         <v>1144</v>
       </c>
-      <c r="B119" s="1">
+      <c r="B119" s="3">
         <v>46170</v>
       </c>
       <c r="C119" t="s">
@@ -12096,7 +12099,7 @@
       <c r="A120">
         <v>1058</v>
       </c>
-      <c r="B120" s="1">
+      <c r="B120" s="3">
         <v>46171</v>
       </c>
       <c r="C120" t="s">
@@ -12151,7 +12154,7 @@
       <c r="A121">
         <v>1097</v>
       </c>
-      <c r="B121" s="1">
+      <c r="B121" s="3">
         <v>46174</v>
       </c>
       <c r="C121" t="s">
@@ -12206,7 +12209,7 @@
       <c r="A122">
         <v>1100</v>
       </c>
-      <c r="B122" s="1">
+      <c r="B122" s="3">
         <v>46175</v>
       </c>
       <c r="C122" t="s">
@@ -12261,7 +12264,7 @@
       <c r="A123">
         <v>1141</v>
       </c>
-      <c r="B123" s="1">
+      <c r="B123" s="3">
         <v>46175</v>
       </c>
       <c r="C123" t="s">
@@ -12316,7 +12319,7 @@
       <c r="A124">
         <v>1134</v>
       </c>
-      <c r="B124" s="1">
+      <c r="B124" s="3">
         <v>46177</v>
       </c>
       <c r="C124" t="s">
@@ -12371,7 +12374,7 @@
       <c r="A125">
         <v>1110</v>
       </c>
-      <c r="B125" s="1">
+      <c r="B125" s="3">
         <v>46179</v>
       </c>
       <c r="C125" t="s">
@@ -12426,7 +12429,7 @@
       <c r="A126">
         <v>1140</v>
       </c>
-      <c r="B126" s="1">
+      <c r="B126" s="3">
         <v>46179</v>
       </c>
       <c r="C126" t="s">
@@ -12481,7 +12484,7 @@
       <c r="A127">
         <v>1069</v>
       </c>
-      <c r="B127" s="1">
+      <c r="B127" s="3">
         <v>46181</v>
       </c>
       <c r="C127" t="s">
@@ -12536,7 +12539,7 @@
       <c r="A128">
         <v>1120</v>
       </c>
-      <c r="B128" s="1">
+      <c r="B128" s="3">
         <v>46181</v>
       </c>
       <c r="C128" t="s">
@@ -12591,7 +12594,7 @@
       <c r="A129">
         <v>1136</v>
       </c>
-      <c r="B129" s="1">
+      <c r="B129" s="3">
         <v>46181</v>
       </c>
       <c r="C129" t="s">
@@ -12646,7 +12649,7 @@
       <c r="A130">
         <v>1039</v>
       </c>
-      <c r="B130" s="1">
+      <c r="B130" s="3">
         <v>46182</v>
       </c>
       <c r="C130" t="s">
@@ -12701,7 +12704,7 @@
       <c r="A131">
         <v>1106</v>
       </c>
-      <c r="B131" s="1">
+      <c r="B131" s="3">
         <v>46182</v>
       </c>
       <c r="C131" t="s">
@@ -12756,7 +12759,7 @@
       <c r="A132">
         <v>1111</v>
       </c>
-      <c r="B132" s="1">
+      <c r="B132" s="3">
         <v>46182</v>
       </c>
       <c r="C132" t="s">
@@ -12811,7 +12814,7 @@
       <c r="A133">
         <v>1145</v>
       </c>
-      <c r="B133" s="1">
+      <c r="B133" s="3">
         <v>46182</v>
       </c>
       <c r="C133" t="s">
@@ -12866,7 +12869,7 @@
       <c r="A134">
         <v>1092</v>
       </c>
-      <c r="B134" s="1">
+      <c r="B134" s="3">
         <v>46183</v>
       </c>
       <c r="C134" t="s">
@@ -12921,7 +12924,7 @@
       <c r="A135">
         <v>1084</v>
       </c>
-      <c r="B135" s="1">
+      <c r="B135" s="3">
         <v>46184</v>
       </c>
       <c r="C135" t="s">
@@ -12976,7 +12979,7 @@
       <c r="A136">
         <v>1020</v>
       </c>
-      <c r="B136" s="1">
+      <c r="B136" s="3">
         <v>46185</v>
       </c>
       <c r="C136" t="s">
@@ -13031,7 +13034,7 @@
       <c r="A137">
         <v>1103</v>
       </c>
-      <c r="B137" s="1">
+      <c r="B137" s="3">
         <v>46185</v>
       </c>
       <c r="C137" t="s">
@@ -13086,7 +13089,7 @@
       <c r="A138">
         <v>1089</v>
       </c>
-      <c r="B138" s="1">
+      <c r="B138" s="3">
         <v>46186</v>
       </c>
       <c r="C138" t="s">
@@ -13141,7 +13144,7 @@
       <c r="A139">
         <v>1001</v>
       </c>
-      <c r="B139" s="1">
+      <c r="B139" s="3">
         <v>46187</v>
       </c>
       <c r="C139" t="s">
@@ -13196,7 +13199,7 @@
       <c r="A140">
         <v>1033</v>
       </c>
-      <c r="B140" s="1">
+      <c r="B140" s="3">
         <v>46191</v>
       </c>
       <c r="C140" t="s">
@@ -13251,7 +13254,7 @@
       <c r="A141">
         <v>1130</v>
       </c>
-      <c r="B141" s="1">
+      <c r="B141" s="3">
         <v>46191</v>
       </c>
       <c r="C141" t="s">
@@ -13306,7 +13309,7 @@
       <c r="A142">
         <v>1148</v>
       </c>
-      <c r="B142" s="1">
+      <c r="B142" s="3">
         <v>46191</v>
       </c>
       <c r="C142" t="s">
@@ -13361,7 +13364,7 @@
       <c r="A143">
         <v>1061</v>
       </c>
-      <c r="B143" s="1">
+      <c r="B143" s="3">
         <v>46193</v>
       </c>
       <c r="C143" t="s">
@@ -13416,7 +13419,7 @@
       <c r="A144">
         <v>1122</v>
       </c>
-      <c r="B144" s="1">
+      <c r="B144" s="3">
         <v>46193</v>
       </c>
       <c r="C144" t="s">
@@ -13471,7 +13474,7 @@
       <c r="A145">
         <v>1045</v>
       </c>
-      <c r="B145" s="1">
+      <c r="B145" s="3">
         <v>46195</v>
       </c>
       <c r="C145" t="s">
@@ -13526,7 +13529,7 @@
       <c r="A146">
         <v>1143</v>
       </c>
-      <c r="B146" s="1">
+      <c r="B146" s="3">
         <v>46195</v>
       </c>
       <c r="C146" t="s">
@@ -13581,7 +13584,7 @@
       <c r="A147">
         <v>1050</v>
       </c>
-      <c r="B147" s="1">
+      <c r="B147" s="3">
         <v>46196</v>
       </c>
       <c r="C147" t="s">
@@ -13636,7 +13639,7 @@
       <c r="A148">
         <v>1115</v>
       </c>
-      <c r="B148" s="1">
+      <c r="B148" s="3">
         <v>46196</v>
       </c>
       <c r="C148" t="s">
@@ -13691,7 +13694,7 @@
       <c r="A149">
         <v>1116</v>
       </c>
-      <c r="B149" s="1">
+      <c r="B149" s="3">
         <v>46196</v>
       </c>
       <c r="C149" t="s">
@@ -13746,7 +13749,7 @@
       <c r="A150">
         <v>1121</v>
       </c>
-      <c r="B150" s="1">
+      <c r="B150" s="3">
         <v>46199</v>
       </c>
       <c r="C150" t="s">
@@ -13801,7 +13804,7 @@
       <c r="A151">
         <v>1109</v>
       </c>
-      <c r="B151" s="1">
+      <c r="B151" s="3">
         <v>46203</v>
       </c>
       <c r="C151" t="s">
@@ -13854,8 +13857,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>